<commit_message>
setup para o início do semestre 2026.2
</commit_message>
<xml_diff>
--- a/plano-de-aulas.xlsx
+++ b/plano-de-aulas.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
     <t>Data</t>
   </si>
@@ -36,7 +36,7 @@
     <t xml:space="preserve"> Programação/Atividades </t>
   </si>
   <si>
-    <t>09-Fev</t>
+    <t>10-Ago</t>
   </si>
   <si>
     <t xml:space="preserve">Introdução à Inteligência Artificial</t>
@@ -54,7 +54,7 @@
     <t xml:space="preserve">Dinâmica em grupo. Referência: Cap 1 e 2 do AIMA e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>11-Fev</t>
+    <t>12-Ago</t>
   </si>
   <si>
     <t xml:space="preserve">O que é agente autônomo? O que são propriedades de ambiente e como isto impacta o desenvolvimento de agentes autônomos? </t>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">Dinâmica em grupo. Referências: Cap 1 e 2 do AIMA e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>23-Fev</t>
+    <t>17-Ago</t>
   </si>
   <si>
     <t xml:space="preserve">Algoritmos de busca cegos</t>
@@ -84,7 +84,7 @@
     <t xml:space="preserve"> Aula expositiva com resolução de exercícios. Referências: Cap 3 e 4 do AIMA e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>25-Fev</t>
+    <t>19-Ago</t>
   </si>
   <si>
     <t xml:space="preserve"> Como um agente encontra uma sequência de ações? Quais são os algoritmos que podemos utilizar? Em que cenário utilizar qual algoritmo? </t>
@@ -96,13 +96,13 @@
     <t xml:space="preserve"> Implementação dos algoritmos de busca e dos agentes autônomos em Python para resolver alguns problemas clássicos da literatura. </t>
   </si>
   <si>
-    <t>02-Mar</t>
-  </si>
-  <si>
-    <t>04-Mar</t>
-  </si>
-  <si>
-    <t>09-Mar</t>
+    <t>24-Ago</t>
+  </si>
+  <si>
+    <t>26-Ago</t>
+  </si>
+  <si>
+    <t>31-Ago</t>
   </si>
   <si>
     <t xml:space="preserve">Algoritmos de busca informados</t>
@@ -117,16 +117,16 @@
     <t xml:space="preserve">Implementação dos algoritmos de busca e dos agentes autônomos em Python para resolver alguns problemas clássicos da literatura. </t>
   </si>
   <si>
-    <t>11-Mar</t>
-  </si>
-  <si>
-    <t>16-Mar</t>
+    <t>2-Set</t>
+  </si>
+  <si>
+    <t>9-Set</t>
   </si>
   <si>
     <t xml:space="preserve">  </t>
   </si>
   <si>
-    <t>18-Mar</t>
+    <t>14-Set</t>
   </si>
   <si>
     <t xml:space="preserve">Como unir todos os conceitos e ferramentas apresentados para resolver um problema complexo? </t>
@@ -141,7 +141,25 @@
     <t xml:space="preserve"> Desenvolvimento de projeto. Referências: Cap 1, 2, 3 e 4 do AIMA e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>23-Mar</t>
+    <t>16-Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambientes competitivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como desenvolver um agente autônomo capaz de identificar estados que satisfazem determinadas restrições? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constraint Satisfaction Problems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementação de um agente autônomo capaz de identificar estados que satisfazem determinadas restrições.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referências: Cap 5 do AIMA e material fornecido pelo professor.</t>
+  </si>
+  <si>
+    <t>21-Set</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS&lt;/strong&gt;</t>
@@ -150,28 +168,10 @@
     <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS - Prova Intermediária&lt;/strong&gt;</t>
   </si>
   <si>
-    <t>25-Mar</t>
-  </si>
-  <si>
-    <t>30-Mar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambientes competitivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como desenvolver um agente autônomo capaz de identificar estados que satisfazem determinadas restrições? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constraint Satisfaction Problems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementação de um agente autônomo capaz de identificar estados que satisfazem determinadas restrições.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referências: Cap 5 do AIMA e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>01-Abr</t>
+    <t>23-Set</t>
+  </si>
+  <si>
+    <t>28-Set</t>
   </si>
   <si>
     <t xml:space="preserve">Como desenvolver um agente autônomo para atuar em ambiente competitivo de soma zero e sem variável aleatória? </t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve"> Aula expositiva com resolução de exercícios e desenvolvimento de projeto. Referências: Cap 6 do AIMA e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>06-Abr</t>
+    <t>30-Set</t>
   </si>
   <si>
     <t xml:space="preserve">Projeto Intermediário</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">Desenvolvimento de projeto em sala de aula</t>
   </si>
   <si>
-    <t>08-Abr</t>
+    <t>5-Out</t>
   </si>
   <si>
     <t xml:space="preserve">Aprendendo políticas</t>
@@ -216,7 +216,7 @@
     <t xml:space="preserve"> Discussão em sala. Exercícios em sala de aula envolvendo o ambiente OpenAI Gym.  Implementação de agentes autônomos usando o algoritmo Q-Learning.</t>
   </si>
   <si>
-    <t>13-Abr</t>
+    <t>7-Out</t>
   </si>
   <si>
     <t xml:space="preserve">Hiper-parâmetros do algoritmo Q-Learning</t>
@@ -231,7 +231,7 @@
     <t xml:space="preserve">Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>15-Abr</t>
+    <t>14-Out</t>
   </si>
   <si>
     <t xml:space="preserve">SARSA: um exemplo de algoritmo on-policy</t>
@@ -246,7 +246,7 @@
     <t xml:space="preserve"> Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
   </si>
   <si>
-    <t>22-Abr</t>
+    <t>19-Out</t>
   </si>
   <si>
     <t xml:space="preserve">Trabalhando com ambientes não-determinísticos</t>
@@ -258,10 +258,10 @@
     <t xml:space="preserve"> Implementação de agentes autônomos usando o algoritmo Q-Learning e Sarsa</t>
   </si>
   <si>
-    <t>27-Abr</t>
-  </si>
-  <si>
-    <t>29-Abr</t>
+    <t>21-Out</t>
+  </si>
+  <si>
+    <t>26-Out</t>
   </si>
   <si>
     <t>Robótica</t>
@@ -273,7 +273,7 @@
     <t xml:space="preserve">Aula expositiva com discussão sobre o assunto.</t>
   </si>
   <si>
-    <t>04-Mai</t>
+    <t>28-Out</t>
   </si>
   <si>
     <t xml:space="preserve">Como unir todos os conceitos e ferramentas apresentados para desenvolver um agente robótico? </t>
@@ -288,16 +288,7 @@
     <t xml:space="preserve">Desenvolvimento de projeto</t>
   </si>
   <si>
-    <t>06-Mai</t>
-  </si>
-  <si>
-    <t>11-Mai</t>
-  </si>
-  <si>
     <t xml:space="preserve">&lt;strong&gt;Avaliação Final da disciplina&lt;/strong&gt;</t>
-  </si>
-  <si>
-    <t>13-Mai</t>
   </si>
 </sst>
 </file>
@@ -348,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -381,6 +372,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" quotePrefix="1">
@@ -1133,57 +1127,56 @@
       <c r="A12" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="7" t="s">
+      <c r="B12" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="C12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="2"/>
     </row>
     <row r="13" s="2" customFormat="1" ht="63" customHeight="1">
       <c r="A13" s="11" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="7" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="G13" s="3"/>
     </row>
     <row r="14" s="2" customFormat="1" ht="63" customHeight="1">
-      <c r="A14" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="A14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="D14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="G14" s="3"/>
     </row>
     <row r="15" s="2" customFormat="1" ht="63" customHeight="1">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="13" t="s">
         <v>51</v>
       </c>
       <c r="B15" s="9"/>
@@ -1202,7 +1195,7 @@
       <c r="G15" s="3"/>
     </row>
     <row r="16" s="2" customFormat="1" ht="63" customHeight="1">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="13" t="s">
         <v>56</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1242,7 +1235,7 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" s="2" customFormat="1" ht="48.75" customHeight="1">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="14" t="s">
         <v>66</v>
       </c>
       <c r="B18" s="8"/>
@@ -1261,7 +1254,7 @@
       <c r="G18" s="3"/>
     </row>
     <row r="19" s="2" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="14" t="s">
         <v>71</v>
       </c>
       <c r="B19" s="3"/>
@@ -1280,7 +1273,7 @@
       <c r="G19" s="3"/>
     </row>
     <row r="20" s="2" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>76</v>
       </c>
       <c r="B20" s="1"/>
@@ -1299,7 +1292,7 @@
       <c r="G20" s="3"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="14" t="s">
         <v>80</v>
       </c>
       <c r="B21" s="1"/>
@@ -1339,7 +1332,7 @@
       <c r="G22" s="1"/>
     </row>
     <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>85</v>
       </c>
       <c r="B23" s="1"/>
@@ -1358,8 +1351,8 @@
       <c r="G23" s="1"/>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="12" t="s">
-        <v>90</v>
+      <c r="A24" s="13">
+        <v>46330</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="3" t="s">
@@ -1377,45 +1370,45 @@
       <c r="G24" s="1"/>
     </row>
     <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="12" t="s">
-        <v>91</v>
+      <c r="A25" s="11">
+        <v>46335</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G25" s="1"/>
     </row>
     <row r="26" s="2" customFormat="1" ht="60.75" customHeight="1">
-      <c r="A26" s="12" t="s">
-        <v>93</v>
+      <c r="A26" s="11">
+        <v>46337</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G26" s="3"/>
     </row>
     <row r="27" s="2" customFormat="1" ht="63" customHeight="1">
-      <c r="A27" s="12"/>
+      <c r="A27" s="13"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" s="2" customFormat="1" ht="48.75" customHeight="1">

</xml_diff>

<commit_message>
publicando material sobre busca heuristica e exercício para APS02
</commit_message>
<xml_diff>
--- a/plano-de-aulas.xlsx
+++ b/plano-de-aulas.xlsx
@@ -129,6 +129,156 @@
     <t>14-Set</t>
   </si>
   <si>
+    <t xml:space="preserve">Ambientes competitivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como desenvolver um agente autônomo capaz de identificar estados que satisfazem determinadas restrições? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constraint Satisfaction Problems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementação de um agente autônomo capaz de identificar estados que satisfazem determinadas restrições.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referências: Cap 5 do AIMA e material fornecido pelo professor.</t>
+  </si>
+  <si>
+    <t>16-Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como desenvolver um agente autônomo para atuar em ambiente competitivo de soma zero e sem variável aleatória? </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jogos de tabuleiro, busca competitiva, algoritmo min-max e função de utilidade. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Implementação de um agente autônomo que deverá atuar em um ambiente competitivo, determinístico e completamente observável. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Aula expositiva com resolução de exercícios e desenvolvimento de projeto. Referências: Cap 6 do AIMA e material fornecido pelo professor.</t>
+  </si>
+  <si>
+    <t>21-Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS&lt;/strong&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS - Prova Intermediária&lt;/strong&gt;</t>
+  </si>
+  <si>
+    <t>23-Set</t>
+  </si>
+  <si>
+    <t>28-Set</t>
+  </si>
+  <si>
+    <t>Robótica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visão geral sobre robótica e framework ROS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aula expositiva com discussão sobre o assunto.</t>
+  </si>
+  <si>
+    <t>30-Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como unir todos os conceitos e ferramentas apresentados para desenvolver um agente robótico? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desenvolvimento de um agente robótico (físico).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementação de um projeto envolvendo um robô físico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desenvolvimento de projeto</t>
+  </si>
+  <si>
+    <t>5-Out</t>
+  </si>
+  <si>
+    <t>7-Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprendendo políticas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O que é aprendizagem por reforço? Qual a sua relação com o desenvolvimento de agentes autônomos? Algoritmo Q-Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definição de aprendizagem por reforço, política de controle e algoritmo Q-Learning. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Discussão em sala. Exercícios em sala de aula envolvendo o ambiente OpenAI Gym.  Implementação de agentes autônomos usando o algoritmo Q-Learning.</t>
+  </si>
+  <si>
+    <t>14-Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiper-parâmetros do algoritmo Q-Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Algoritmo Q-Learning: detalhes e hiperparâmetros. Apresentação do ambiente OpenAI Gym. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exercícios em sala de aula envolvendo o ambiente OpenAI Gym.  Implementação de agentes autônomos usando o algoritmo Q-Learning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
+  </si>
+  <si>
+    <t>19-Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SARSA: um exemplo de algoritmo on-policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Algoritmo Q-Learning: detalhes e hiperparâmetros. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementação de agentes autônomos usando o algoritmo Sarsa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
+  </si>
+  <si>
+    <t>21-Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trabalhando com ambientes não-determinísticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambientes não-determinísticos. Reinforcement Learning: métodos tabulares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Implementação de agentes autônomos usando o algoritmo Q-Learning e Sarsa</t>
+  </si>
+  <si>
+    <t>26-Out</t>
+  </si>
+  <si>
+    <t>28-Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projeto Final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tema a ser definido</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Desenvolvimento de um agente autônomo que atua em um ambiente discreto, determinístico, síncrono, simulado e *single agent* ou *multi-agent*. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desenvolvimento de projeto em sala de aula</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Desenvolvimento de projeto. Referências: Cap 1, 2, 3, 4 e 21 do AIMA Cap. 18 do Géron e material fornecido pelo professor.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Como unir todos os conceitos e ferramentas apresentados para resolver um problema complexo? </t>
   </si>
   <si>
@@ -136,156 +286,6 @@
   </si>
   <si>
     <t xml:space="preserve"> Implementação de um projeto, provavelmente, envolvendo algum framework de simulação (i.e., Gym Open AI). </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Desenvolvimento de projeto. Referências: Cap 1, 2, 3 e 4 do AIMA e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>16-Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambientes competitivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como desenvolver um agente autônomo capaz de identificar estados que satisfazem determinadas restrições? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constraint Satisfaction Problems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementação de um agente autônomo capaz de identificar estados que satisfazem determinadas restrições.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referências: Cap 5 do AIMA e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>21-Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS&lt;/strong&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;strong&gt;SEMANA DE PROVAS - Prova Intermediária&lt;/strong&gt;</t>
-  </si>
-  <si>
-    <t>23-Set</t>
-  </si>
-  <si>
-    <t>28-Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como desenvolver um agente autônomo para atuar em ambiente competitivo de soma zero e sem variável aleatória? </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Jogos de tabuleiro, busca competitiva, algoritmo min-max e função de utilidade. </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Implementação de um agente autônomo que deverá atuar em um ambiente competitivo, determinístico e completamente observável. </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Aula expositiva com resolução de exercícios e desenvolvimento de projeto. Referências: Cap 6 do AIMA e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>30-Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projeto Intermediário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tema a ser definido</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Desenvolvimento de um agente autônomo que atua em um ambiente discreto, determinístico, síncrono, simulado e *single agent* ou *multi-agent*. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desenvolvimento de projeto em sala de aula</t>
-  </si>
-  <si>
-    <t>5-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aprendendo políticas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O que é aprendizagem por reforço? Qual a sua relação com o desenvolvimento de agentes autônomos? Algoritmo Q-Learning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definição de aprendizagem por reforço, política de controle e algoritmo Q-Learning. </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Discussão em sala. Exercícios em sala de aula envolvendo o ambiente OpenAI Gym.  Implementação de agentes autônomos usando o algoritmo Q-Learning.</t>
-  </si>
-  <si>
-    <t>7-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiper-parâmetros do algoritmo Q-Learning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Algoritmo Q-Learning: detalhes e hiperparâmetros. Apresentação do ambiente OpenAI Gym. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exercícios em sala de aula envolvendo o ambiente OpenAI Gym.  Implementação de agentes autônomos usando o algoritmo Q-Learning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>14-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SARSA: um exemplo de algoritmo on-policy</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Algoritmo Q-Learning: detalhes e hiperparâmetros. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementação de agentes autônomos usando o algoritmo Sarsa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Aula expositiva com resolução de exercícios. Referências: Cap 21 do AIMA, Cap. 18 do Géron e material fornecido pelo professor.</t>
-  </si>
-  <si>
-    <t>19-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trabalhando com ambientes não-determinísticos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambientes não-determinísticos. Reinforcement Learning: métodos tabulares</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Implementação de agentes autônomos usando o algoritmo Q-Learning e Sarsa</t>
-  </si>
-  <si>
-    <t>21-Out</t>
-  </si>
-  <si>
-    <t>26-Out</t>
-  </si>
-  <si>
-    <t>Robótica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visão geral sobre robótica e framework ROS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aula expositiva com discussão sobre o assunto.</t>
-  </si>
-  <si>
-    <t>28-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como unir todos os conceitos e ferramentas apresentados para desenvolver um agente robótico? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desenvolvimento de um agente robótico (físico).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implementação de um projeto envolvendo um robô físico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desenvolvimento de projeto</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;strong&gt;Avaliação Final da disciplina&lt;/strong&gt;</t>
@@ -339,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -381,6 +381,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1108,26 +1111,25 @@
       <c r="A11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="1"/>
+      <c r="B11" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G11" s="3"/>
     </row>
     <row r="12" s="2" customFormat="1" ht="63" customHeight="1">
       <c r="A12" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" s="7" t="s">
         <v>42</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1179,112 +1181,113 @@
       <c r="A15" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="9"/>
+      <c r="B15" s="7" t="s">
+        <v>52</v>
+      </c>
       <c r="C15" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="G15" s="3"/>
     </row>
     <row r="16" s="2" customFormat="1" ht="63" customHeight="1">
       <c r="A16" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="E16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" s="1"/>
       <c r="G16" s="3"/>
     </row>
     <row r="17" s="2" customFormat="1" ht="63" customHeight="1">
       <c r="A17" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G17" s="3"/>
     </row>
     <row r="18" s="2" customFormat="1" ht="48.75" customHeight="1">
       <c r="A18" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B18" s="8"/>
+        <v>61</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>62</v>
+      </c>
       <c r="C18" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="G18" s="3"/>
     </row>
     <row r="19" s="2" customFormat="1" ht="49.5" customHeight="1">
       <c r="A19" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="3"/>
+        <v>66</v>
+      </c>
+      <c r="B19" s="8"/>
       <c r="C19" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G19" s="3"/>
     </row>
     <row r="20" s="2" customFormat="1" ht="49.5" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="B20" s="3"/>
       <c r="C20" s="3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>75</v>
@@ -1293,7 +1296,7 @@
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="3" t="s">
@@ -1312,41 +1315,41 @@
     </row>
     <row r="22" ht="37.5" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>82</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="B22" s="1"/>
       <c r="C22" s="3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="G22" s="1"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="G23" s="1"/>
     </row>
@@ -1356,16 +1359,16 @@
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="G24" s="1"/>
     </row>
@@ -1409,6 +1412,7 @@
     </row>
     <row r="27" s="2" customFormat="1" ht="63" customHeight="1">
       <c r="A27" s="13"/>
+      <c r="B27" s="2"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" s="2" customFormat="1" ht="48.75" customHeight="1">

</xml_diff>